<commit_message>
docs(mock): update flow_mock_excel.xlsx with notification and log flows, update ApiGateway submodule pointer
</commit_message>
<xml_diff>
--- a/docs/excel/flow_mock_excel.xlsx
+++ b/docs/excel/flow_mock_excel.xlsx
@@ -2085,8 +2085,8 @@
       <c r="E4" s="15" t="inlineStr">
         <is>
           <t>{
-"email": "string",
-"otp_code": "string: 6 digits"
+  "email": "user@example.com",
+  "otp": "123456"
 }</t>
         </is>
       </c>
@@ -2459,10 +2459,10 @@
       <c r="E9" s="10" t="inlineStr">
         <is>
           <t>{
-"email": "string",
-"otp_code": "string: 6 digits",
-"new_password": "string",
-"confirm_password": "string"
+  "email": "user@example.com",
+  "otpCode": "123456",
+  "newPassword": "NewPassword123@",
+  "confirmPassword": "NewPassword123@"
 }</t>
         </is>
       </c>
@@ -2969,19 +2969,19 @@
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Body:
 {
-"username": "string (optional, max 100)",
-"first_name": "string",
-"last_name": "string",
-"phone_number": "string",
-"address": {
-"province_id": "int",
-"district_id": "int",
-"ward_code": "string",
-"street_address": "string"
-}
+  "username": "string (optional, max 100)",
+  "firstName": "string",
+  "lastName": "string",
+  "phoneNumber": "string",
+  "address": {
+    "provinceId": 1,
+    "districtId": 1,
+    "wardCode": "001",
+    "streetAddress": "string"
+  }
 }</t>
         </is>
       </c>
@@ -3940,15 +3940,15 @@
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Body:
 {
-"transaction_type": "string (\"ORDER\" | \"AUCTION\")",
-"transaction_id": "uuid",
-"target_user_id": "uuid",
-"rating": "int (1..5)",
-"comment": "string (10..500 ký tự)",
-"media_urls": "string[] (optional)"
+  "transactionType": "ORDER|AUCTION",
+  "transactionId": "uuid",
+  "targetUserId": "uuid",
+  "rating": 5,
+  "comment": "Giao hang nhanh, dong goi can than.",
+  "mediaUrls": ["https://img.example.com/review1.png"]
 }</t>
         </is>
       </c>
@@ -4119,13 +4119,13 @@
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Body:
 {
-"reported_user_id": "uuid",
-"violation_type": "string",
-"description": "string (10..1000 ký tự)",
-"evidence_urls": "string[] (optional)"
+  "reportedUserId": "uuid",
+  "violationType": "SPAM|FRAUD|INAPPROPRIATE_CONTENT",
+  "description": "Nguoi dung co hanh vi gian lan.",
+  "evidenceUrls": ["https://img.example.com/evidence1.png"]
 }</t>
         </is>
       </c>
@@ -4286,19 +4286,19 @@
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Body:
 {
-"shopName": "string",
-"businessEmail": "string",
-"hotline": "string",
-"warehouseAddress": {
-"province_id": "int",
-"district_id": "int",
-"ward_code": "string",
-"street_address": "string"
-},
-"identityCardNumber": "string"
+  "shopName": "string",
+  "businessEmail": "string",
+  "hotline": "string",
+  "warehouseAddress": {
+    "provinceId": 1,
+    "districtId": 1,
+    "wardCode": "001",
+    "streetAddress": "string"
+  },
+  "identityCardNumber": "string"
 }</t>
         </is>
       </c>
@@ -4752,18 +4752,18 @@
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Body:
 {
-"shopName": "string (optional)",
-"hotline": "string (optional)",
-"pickupAddress": {
-"province_id": "int",
-"district_id": "int",
-"ward_code": "string",
-"street_address": "string"
-},
-"description": "string"
+  "shopName": "string",
+  "hotline": "string",
+  "pickupAddress": {
+    "provinceId": 1,
+    "districtId": 1,
+    "wardCode": "001",
+    "streetAddress": "string"
+  },
+  "description": "string"
 }</t>
         </is>
       </c>
@@ -5183,13 +5183,13 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Query:
 {
-"page": "int (default: 1)",
-"limit": "int (default: 20)",
-"status": "string (optional)",
-"violation_type": "string (optional)"
+  "page": 1,
+  "limit": 20,
+  "status": "PENDING|RESOLVED|DISMISSED",
+  "violationType": "SPAM|FRAUD"
 }</t>
         </is>
       </c>
@@ -6186,17 +6186,13 @@
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Path: { "userId": "uuid" }
 Body:
 {
-"role_codes": [
-"STAFF"
-],
-"role_ids": [
-1
-],
-"reason": "string"
+  "roleCodes": ["Staff"],
+  "roleIds": [1],
+  "reason": "Promotion to customer support staff."
 }</t>
         </is>
       </c>
@@ -6505,12 +6501,12 @@
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
-Path: { "roleId": "int" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
+Path: { "roleId": 1 }
 Body:
 {
-"description": "string",
-"permission_ids": "int[]"
+  "description": "Customer support and complaint resolution.",
+  "permissionIds": [1, 2, 3]
 }</t>
         </is>
       </c>
@@ -6579,44 +6575,45 @@
       </c>
       <c r="E60" s="15" t="inlineStr">
         <is>
-          <t>Headers: { "Authorization": "Bearer JWT" }
+          <t>Headers: { "Authorization": "Bearer &lt;JWT&gt;" }
 Query:
 {
-"page": "int (default: 1)",
-"limit": "int (default: 20)",
-"actor_id": "uuid (optional)",
-"action": "string (optional)",
-"from_date": "datetime (optional)",
-"to_date": "datetime (optional)"
+  "page": 1,
+  "limit": 20,
+  "actorId": "uuid",
+  "action": "string",
+  "fromDate": "2026-10-01T00:00:00Z",
+  "toDate": "2026-10-26T00:00:00Z"
 }</t>
         </is>
       </c>
       <c r="F60" s="15" t="inlineStr">
         <is>
-          <t>{
-"msg": "Lấy nhật ký kiểm toán thành công",
-"data": {
-"items": [
+          <t>200 OK:
 {
-"id": "uuid",
-"actorId": "uuid",
-"action": "string",
-"targetEntity": "string",
-"oldValues": "object",
-"newValues": "object",
-"reason": "string",
-"ipAddress": "string",
-"createdAt": "timestamp"
-}
-]
-}
+  "items": [
+    {
+      "id": "uuid",
+      "actorId": "uuid",
+      "action": "USER_BANNED",
+      "targetEntity": "users",
+      "oldValues": {},
+      "newValues": {},
+      "reason": "Policy violation.",
+      "ipAddress": "127.0.0.1",
+      "createdAt": "2026-10-26T00:00:00Z"
+    }
+  ],
+  "total": 1,
+  "page": 1,
+  "limit": 20
 }</t>
         </is>
       </c>
       <c r="G60" s="15" t="inlineStr">
         <is>
-          <t>- [401] ERR_UNAUTHORIZED: Chưa đăng nhập
-- [403] ERR_PERMISSION_DENIED: Không có quyền tra cứu nhật ký kiểm toán (audit:view)</t>
+          <t>401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have permission to view audit logs.</t>
         </is>
       </c>
       <c r="H60" s="84" t="n"/>
@@ -6999,7 +6996,11 @@
 }</t>
         </is>
       </c>
-      <c r="G66" s="18" t="n"/>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_PAGE: Page and pageSize must be positive integers.</t>
+        </is>
+      </c>
       <c r="H66" s="30" t="n"/>
       <c r="I66" s="8" t="inlineStr">
         <is>
@@ -7082,7 +7083,11 @@
 }</t>
         </is>
       </c>
-      <c r="G67" s="34" t="n"/>
+      <c r="G67" s="34" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_FILTER: Search filter parameters are invalid.</t>
+        </is>
+      </c>
       <c r="H67" s="30" t="n"/>
       <c r="I67" s="32" t="inlineStr">
         <is>
@@ -7178,7 +7183,12 @@
 }</t>
         </is>
       </c>
-      <c r="G68" s="18" t="n"/>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_PRODUCT_ID: Product ID format is invalid.
+404 PRODUCT_NOT_FOUND: Product was not found or is inactive.</t>
+        </is>
+      </c>
       <c r="H68" s="30" t="n"/>
       <c r="I68" s="8" t="inlineStr">
         <is>
@@ -15353,13 +15363,57 @@
     </row>
     <row r="185" ht="15.75" customHeight="1" s="81">
       <c r="A185" s="9" t="n"/>
-      <c r="B185" s="9" t="n"/>
-      <c r="C185" s="21" t="n"/>
-      <c r="D185" s="21" t="n"/>
-      <c r="E185" s="21" t="n"/>
-      <c r="F185" s="21" t="n"/>
-      <c r="G185" s="21" t="n"/>
-      <c r="H185" s="66" t="n"/>
+      <c r="B185" s="9" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C185" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/devices</t>
+        </is>
+      </c>
+      <c r="D185" s="21" t="inlineStr">
+        <is>
+          <t>Đăng ký hoặc làm mới FCM/APNs device token để nhận push notification</t>
+        </is>
+      </c>
+      <c r="E185" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Body:
+{
+  "platform": "WEB|IOS|ANDROID",
+  "token": "string"
+}</t>
+        </is>
+      </c>
+      <c r="F185" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "deviceId": "uuid",
+  "userId": "uuid",
+  "platform": "WEB|IOS|ANDROID",
+  "isActive": true,
+  "lastSeenAt": "2026-10-26T00:00:00Z"
+}</t>
+        </is>
+      </c>
+      <c r="G185" s="21" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_DEVICE_TOKEN: Platform or token is invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.</t>
+        </is>
+      </c>
+      <c r="H185" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-01</t>
+        </is>
+      </c>
       <c r="I185" s="21" t="n"/>
       <c r="J185" s="21" t="n"/>
       <c r="K185" s="21" t="n"/>
@@ -15382,13 +15436,50 @@
     </row>
     <row r="186" ht="15.75" customHeight="1" s="81">
       <c r="A186" s="76" t="n"/>
-      <c r="B186" s="76" t="n"/>
-      <c r="C186" s="77" t="n"/>
-      <c r="D186" s="77" t="n"/>
-      <c r="E186" s="77" t="n"/>
-      <c r="F186" s="77" t="n"/>
-      <c r="G186" s="77" t="n"/>
-      <c r="H186" s="66" t="n"/>
+      <c r="B186" s="76" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C186" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/devices</t>
+        </is>
+      </c>
+      <c r="D186" s="77" t="inlineStr">
+        <is>
+          <t>Thu hồi hoặc vô hiệu hóa device token khi logout hoặc tắt quyền push</t>
+        </is>
+      </c>
+      <c r="E186" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Body:
+{
+  "token": "string"
+}</t>
+        </is>
+      </c>
+      <c r="F186" s="77" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="G186" s="77" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_TOKEN: Token is missing or invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.
+404 DEVICE_TOKEN_NOT_FOUND: Device token was not found for this user.</t>
+        </is>
+      </c>
+      <c r="H186" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-02</t>
+        </is>
+      </c>
       <c r="I186" s="77" t="n"/>
       <c r="J186" s="77" t="n"/>
       <c r="K186" s="77" t="n"/>
@@ -15411,13 +15502,54 @@
     </row>
     <row r="187" ht="15.75" customHeight="1" s="81">
       <c r="A187" s="9" t="n"/>
-      <c r="B187" s="9" t="n"/>
-      <c r="C187" s="21" t="n"/>
-      <c r="D187" s="21" t="n"/>
-      <c r="E187" s="21" t="n"/>
-      <c r="F187" s="21" t="n"/>
-      <c r="G187" s="21" t="n"/>
-      <c r="H187" s="66" t="n"/>
+      <c r="B187" s="9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C187" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/preferences</t>
+        </is>
+      </c>
+      <c r="D187" s="21" t="inlineStr">
+        <is>
+          <t>Lấy danh sách cấu hình bật/tắt nhận thông báo của người dùng</t>
+        </is>
+      </c>
+      <c r="E187" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}</t>
+        </is>
+      </c>
+      <c r="F187" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "items": [
+    {
+      "notificationType": "ORDER_PAID|AUCTION_OUTBID|PROMOTION",
+      "channelCode": "EMAIL|PUSH|IN_APP",
+      "isEnabled": true,
+      "isMandatory": true
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G187" s="21" t="inlineStr">
+        <is>
+          <t>401 UNAUTHORIZED: Token is missing, expired, or invalid.</t>
+        </is>
+      </c>
+      <c r="H187" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-03</t>
+        </is>
+      </c>
       <c r="I187" s="21" t="n"/>
       <c r="J187" s="21" t="n"/>
       <c r="K187" s="21" t="n"/>
@@ -15440,13 +15572,66 @@
     </row>
     <row r="188" ht="15.75" customHeight="1" s="81">
       <c r="A188" s="76" t="n"/>
-      <c r="B188" s="76" t="n"/>
-      <c r="C188" s="77" t="n"/>
-      <c r="D188" s="77" t="n"/>
-      <c r="E188" s="77" t="n"/>
-      <c r="F188" s="77" t="n"/>
-      <c r="G188" s="77" t="n"/>
-      <c r="H188" s="66" t="n"/>
+      <c r="B188" s="76" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="C188" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/preferences</t>
+        </is>
+      </c>
+      <c r="D188" s="77" t="inlineStr">
+        <is>
+          <t>Cập nhật tùy chọn bật/tắt nhận thông báo theo loại sự kiện và kênh gửi</t>
+        </is>
+      </c>
+      <c r="E188" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Body:
+{
+  "preferences": [
+    {
+      "notificationType": "ORDER_PAID",
+      "channelCode": "EMAIL",
+      "isEnabled": true
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="F188" s="77" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "updatedCount": 1,
+  "preferences": [
+    {
+      "notificationType": "ORDER_PAID",
+      "channelCode": "EMAIL",
+      "isEnabled": true
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G188" s="77" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_PREFERENCES: Notification type or channel code is invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.
+422 MANDATORY_NOTIFICATION_CANNOT_DISABLE: Mandatory security or transaction notification cannot be disabled.</t>
+        </is>
+      </c>
+      <c r="H188" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-04</t>
+        </is>
+      </c>
       <c r="I188" s="77" t="n"/>
       <c r="J188" s="77" t="n"/>
       <c r="K188" s="77" t="n"/>
@@ -15469,13 +15654,71 @@
     </row>
     <row r="189" ht="15.75" customHeight="1" s="81">
       <c r="A189" s="9" t="n"/>
-      <c r="B189" s="9" t="n"/>
-      <c r="C189" s="21" t="n"/>
-      <c r="D189" s="21" t="n"/>
-      <c r="E189" s="21" t="n"/>
-      <c r="F189" s="21" t="n"/>
-      <c r="G189" s="21" t="n"/>
-      <c r="H189" s="66" t="n"/>
+      <c r="B189" s="9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C189" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/me</t>
+        </is>
+      </c>
+      <c r="D189" s="21" t="inlineStr">
+        <is>
+          <t>Lấy danh sách lịch sử thông báo in-app (quả chuông) kèm số lượng chưa đọc</t>
+        </is>
+      </c>
+      <c r="E189" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Query:
+{
+  "isRead": false,
+  "notificationType": "ORDER_PAID",
+  "pageIndex": 1,
+  "pageSize": 20
+}</t>
+        </is>
+      </c>
+      <c r="F189" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "unreadCount": 3,
+  "totalCount": 10,
+  "items": [
+    {
+      "id": "uuid",
+      "notificationType": "ORDER_PAID",
+      "title": "Don hang #SUB-01 da duoc thanh toan",
+      "body": "Don hang tri gia 480.000d da duoc thanh toan thanh cong.",
+      "payload": {
+        "orderId": "uuid",
+        "subOrderId": "uuid"
+      },
+      "isRead": false,
+      "readAt": null,
+      "createdAt": "2026-10-26T00:00:00Z"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G189" s="21" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_PAGE: PageIndex or pageSize is invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.</t>
+        </is>
+      </c>
+      <c r="H189" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-05</t>
+        </is>
+      </c>
       <c r="I189" s="21" t="n"/>
       <c r="J189" s="21" t="n"/>
       <c r="K189" s="21" t="n"/>
@@ -15498,13 +15741,54 @@
     </row>
     <row r="190" ht="15.75" customHeight="1" s="81">
       <c r="A190" s="76" t="n"/>
-      <c r="B190" s="76" t="n"/>
-      <c r="C190" s="77" t="n"/>
-      <c r="D190" s="77" t="n"/>
-      <c r="E190" s="77" t="n"/>
-      <c r="F190" s="77" t="n"/>
-      <c r="G190" s="77" t="n"/>
-      <c r="H190" s="66" t="n"/>
+      <c r="B190" s="76" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="C190" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/me/read</t>
+        </is>
+      </c>
+      <c r="D190" s="77" t="inlineStr">
+        <is>
+          <t>Đánh dấu một số hoặc toàn bộ thông báo trong hộp thư là đã đọc</t>
+        </is>
+      </c>
+      <c r="E190" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Body:
+{
+  "notificationIds": ["uuid"],
+  "markAll": false
+}</t>
+        </is>
+      </c>
+      <c r="F190" s="77" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "updatedCount": 1,
+  "unreadCount": 2
+}</t>
+        </is>
+      </c>
+      <c r="G190" s="77" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_INPUT: Notification IDs list is invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.</t>
+        </is>
+      </c>
+      <c r="H190" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-06</t>
+        </is>
+      </c>
       <c r="I190" s="77" t="n"/>
       <c r="J190" s="77" t="n"/>
       <c r="K190" s="77" t="n"/>
@@ -15527,13 +15811,63 @@
     </row>
     <row r="191" ht="15.75" customHeight="1" s="81">
       <c r="A191" s="9" t="n"/>
-      <c r="B191" s="9" t="n"/>
-      <c r="C191" s="21" t="n"/>
-      <c r="D191" s="21" t="n"/>
-      <c r="E191" s="21" t="n"/>
-      <c r="F191" s="21" t="n"/>
-      <c r="G191" s="21" t="n"/>
-      <c r="H191" s="66" t="n"/>
+      <c r="B191" s="9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C191" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/notifications/channels/{code}</t>
+        </is>
+      </c>
+      <c r="D191" s="21" t="inlineStr">
+        <is>
+          <t>Admin xem trạng thái và cấu hình kênh gửi thông báo</t>
+        </is>
+      </c>
+      <c r="E191" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Path:
+{
+  "code": "EMAIL|PUSH|IN_APP|SMS"
+}</t>
+        </is>
+      </c>
+      <c r="F191" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "id": "uuid",
+  "code": "EMAIL",
+  "name": "Email Service",
+  "provider": "SMTP",
+  "config": {
+    "host": "smtp.example.com",
+    "port": 587,
+    "fromAddress": "noreply@shop.example.com"
+  },
+  "isEnabled": true,
+  "updatedAt": "2026-10-26T00:00:00Z"
+}</t>
+        </is>
+      </c>
+      <c r="G191" s="21" t="inlineStr">
+        <is>
+          <t>401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.
+404 CHANNEL_NOT_FOUND: Notification channel code was not found.</t>
+        </is>
+      </c>
+      <c r="H191" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-07</t>
+        </is>
+      </c>
       <c r="I191" s="21" t="n"/>
       <c r="J191" s="21" t="n"/>
       <c r="K191" s="21" t="n"/>
@@ -15556,13 +15890,75 @@
     </row>
     <row r="192" ht="15.75" customHeight="1" s="81">
       <c r="A192" s="76" t="n"/>
-      <c r="B192" s="76" t="n"/>
-      <c r="C192" s="77" t="n"/>
-      <c r="D192" s="77" t="n"/>
-      <c r="E192" s="77" t="n"/>
-      <c r="F192" s="77" t="n"/>
-      <c r="G192" s="77" t="n"/>
-      <c r="H192" s="66" t="n"/>
+      <c r="B192" s="76" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="C192" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/notifications/channels/{code}</t>
+        </is>
+      </c>
+      <c r="D192" s="77" t="inlineStr">
+        <is>
+          <t>Admin cập nhật cấu hình và bật/tắt kênh gửi thông báo</t>
+        </is>
+      </c>
+      <c r="E192" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Path:
+{
+  "code": "EMAIL|PUSH|IN_APP|SMS"
+}
+Body:
+{
+  "name": "Email Service",
+  "provider": "SMTP",
+  "config": {
+    "host": "smtp.example.com",
+    "port": 587,
+    "fromAddress": "noreply@shop.example.com"
+  },
+  "isEnabled": true
+}</t>
+        </is>
+      </c>
+      <c r="F192" s="77" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "id": "uuid",
+  "code": "EMAIL",
+  "name": "Email Service",
+  "provider": "SMTP",
+  "config": {
+    "host": "smtp.example.com",
+    "port": 587,
+    "fromAddress": "noreply@shop.example.com"
+  },
+  "isEnabled": true,
+  "updatedAt": "2026-10-26T00:00:00Z"
+}</t>
+        </is>
+      </c>
+      <c r="G192" s="77" t="inlineStr">
+        <is>
+          <t>400 SECRET_IN_CONFIG_FORBIDDEN: Secrets like passwords or API keys are not allowed in config body.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.
+404 CHANNEL_NOT_FOUND: Notification channel code was not found.</t>
+        </is>
+      </c>
+      <c r="H192" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-07</t>
+        </is>
+      </c>
       <c r="I192" s="77" t="n"/>
       <c r="J192" s="77" t="n"/>
       <c r="K192" s="77" t="n"/>
@@ -15585,13 +15981,65 @@
     </row>
     <row r="193" ht="15.75" customHeight="1" s="81">
       <c r="A193" s="9" t="n"/>
-      <c r="B193" s="9" t="n"/>
-      <c r="C193" s="21" t="n"/>
-      <c r="D193" s="21" t="n"/>
-      <c r="E193" s="21" t="n"/>
-      <c r="F193" s="21" t="n"/>
-      <c r="G193" s="21" t="n"/>
-      <c r="H193" s="66" t="n"/>
+      <c r="B193" s="9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C193" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/notifications/templates</t>
+        </is>
+      </c>
+      <c r="D193" s="21" t="inlineStr">
+        <is>
+          <t>Admin xem danh sách mẫu thông báo (Template Engine)</t>
+        </is>
+      </c>
+      <c r="E193" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Query:
+{
+  "channelCode": "EMAIL",
+  "notificationType": "ORDER_PAID"
+}</t>
+        </is>
+      </c>
+      <c r="F193" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "items": [
+    {
+      "id": "uuid",
+      "code": "ORDER_PAID_EMAIL",
+      "notificationType": "ORDER_PAID",
+      "channelCode": "EMAIL",
+      "subjectTemplate": "Don hang {{orderNo}} thanh toan thanh cong",
+      "bodyTemplate": "&lt;p&gt;Xin chao {{userName}}, don hang {{orderNo}} da duoc xac nhan.&lt;/p&gt;",
+      "isMandatory": true,
+      "locale": "vi-VN",
+      "isActive": true
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G193" s="21" t="inlineStr">
+        <is>
+          <t>401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.</t>
+        </is>
+      </c>
+      <c r="H193" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-08</t>
+        </is>
+      </c>
       <c r="I193" s="21" t="n"/>
       <c r="J193" s="21" t="n"/>
       <c r="K193" s="21" t="n"/>
@@ -15614,13 +16062,67 @@
     </row>
     <row r="194" ht="15.75" customHeight="1" s="81">
       <c r="A194" s="76" t="n"/>
-      <c r="B194" s="76" t="n"/>
-      <c r="C194" s="77" t="n"/>
-      <c r="D194" s="77" t="n"/>
-      <c r="E194" s="77" t="n"/>
-      <c r="F194" s="77" t="n"/>
-      <c r="G194" s="77" t="n"/>
-      <c r="H194" s="66" t="n"/>
+      <c r="B194" s="76" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C194" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/notifications/templates</t>
+        </is>
+      </c>
+      <c r="D194" s="77" t="inlineStr">
+        <is>
+          <t>Admin tạo mẫu nội dung thông báo mới</t>
+        </is>
+      </c>
+      <c r="E194" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Body:
+{
+  "code": "ORDER_PAID_EMAIL",
+  "notificationType": "ORDER_PAID",
+  "channelCode": "EMAIL",
+  "subjectTemplate": "Don hang {{orderNo}} thanh toan thanh cong",
+  "bodyTemplate": "&lt;p&gt;Xin chao {{userName}}, don hang {{orderNo}} da duoc xac nhan.&lt;/p&gt;",
+  "isMandatory": true,
+  "locale": "vi-VN",
+  "isActive": true
+}</t>
+        </is>
+      </c>
+      <c r="F194" s="77" t="inlineStr">
+        <is>
+          <t>201 Created:
+{
+  "id": "uuid",
+  "code": "ORDER_PAID_EMAIL",
+  "notificationType": "ORDER_PAID",
+  "channelCode": "EMAIL",
+  "isMandatory": true,
+  "locale": "vi-VN",
+  "isActive": true
+}</t>
+        </is>
+      </c>
+      <c r="G194" s="77" t="inlineStr">
+        <is>
+          <t>400 INVALID_TEMPLATE_SYNTAX: Template syntax is invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.
+409 TEMPLATE_CODE_DUPLICATED: Template code and locale already exist.</t>
+        </is>
+      </c>
+      <c r="H194" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-08</t>
+        </is>
+      </c>
       <c r="I194" s="77" t="n"/>
       <c r="J194" s="77" t="n"/>
       <c r="K194" s="77" t="n"/>
@@ -15643,13 +16145,75 @@
     </row>
     <row r="195" ht="15.75" customHeight="1" s="81">
       <c r="A195" s="9" t="n"/>
-      <c r="B195" s="9" t="n"/>
-      <c r="C195" s="21" t="n"/>
-      <c r="D195" s="21" t="n"/>
-      <c r="E195" s="21" t="n"/>
-      <c r="F195" s="21" t="n"/>
-      <c r="G195" s="21" t="n"/>
-      <c r="H195" s="66" t="n"/>
+      <c r="B195" s="9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C195" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/notifications</t>
+        </is>
+      </c>
+      <c r="D195" s="21" t="inlineStr">
+        <is>
+          <t>Admin/Staff tra cứu lịch sử gửi thông báo và nhật ký lỗi delivery</t>
+        </is>
+      </c>
+      <c r="E195" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Query:
+{
+  "userId": "uuid",
+  "notificationType": "ORDER_PAID",
+  "status": "COMPLETED|PENDING|FAILED",
+  "pageIndex": 1,
+  "pageSize": 20
+}</t>
+        </is>
+      </c>
+      <c r="F195" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "total": 1,
+  "items": [
+    {
+      "notificationId": "uuid",
+      "userId": "uuid",
+      "notificationType": "ORDER_PAID",
+      "status": "COMPLETED",
+      "createdAt": "2026-10-26T00:00:00Z",
+      "deliveries": [
+        {
+          "deliveryId": "uuid",
+          "channelCode": "EMAIL",
+          "destination": "u***@gmail.com",
+          "status": "SENT",
+          "attemptCount": 1
+        }
+      ]
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G195" s="21" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_FILTER: Query filter parameters are invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.</t>
+        </is>
+      </c>
+      <c r="H195" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-09</t>
+        </is>
+      </c>
       <c r="I195" s="21" t="n"/>
       <c r="J195" s="21" t="n"/>
       <c r="K195" s="21" t="n"/>
@@ -15672,13 +16236,66 @@
     </row>
     <row r="196" ht="15.75" customHeight="1" s="81">
       <c r="A196" s="76" t="n"/>
-      <c r="B196" s="76" t="n"/>
-      <c r="C196" s="77" t="n"/>
-      <c r="D196" s="77" t="n"/>
-      <c r="E196" s="77" t="n"/>
-      <c r="F196" s="77" t="n"/>
-      <c r="G196" s="77" t="n"/>
-      <c r="H196" s="66" t="n"/>
+      <c r="B196" s="76" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C196" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/event-logs</t>
+        </is>
+      </c>
+      <c r="D196" s="77" t="inlineStr">
+        <is>
+          <t>Admin tra cứu nhật ký sự kiện kỹ thuật message bus (90 ngày)</t>
+        </is>
+      </c>
+      <c r="E196" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Query:
+{
+  "sourceService": "Commerce|Auction|User|Wallet",
+  "eventType": "OrderPaid",
+  "pageIndex": 1,
+  "pageSize": 20
+}</t>
+        </is>
+      </c>
+      <c r="F196" s="77" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "total": 1,
+  "items": [
+    {
+      "id": "uuid",
+      "eventId": "uuid",
+      "eventType": "OrderPaid",
+      "sourceService": "Commerce",
+      "actorId": "uuid",
+      "occurredAt": "2026-10-26T00:00:00Z"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G196" s="77" t="inlineStr">
+        <is>
+          <t>400 VAL_INVALID_FILTER: Query date range or filter is invalid.
+401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.</t>
+        </is>
+      </c>
+      <c r="H196" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-13</t>
+        </is>
+      </c>
       <c r="I196" s="77" t="n"/>
       <c r="J196" s="77" t="n"/>
       <c r="K196" s="77" t="n"/>
@@ -15701,13 +16318,63 @@
     </row>
     <row r="197" ht="15.75" customHeight="1" s="81">
       <c r="A197" s="9" t="n"/>
-      <c r="B197" s="9" t="n"/>
-      <c r="C197" s="21" t="n"/>
-      <c r="D197" s="21" t="n"/>
-      <c r="E197" s="21" t="n"/>
-      <c r="F197" s="21" t="n"/>
-      <c r="G197" s="21" t="n"/>
-      <c r="H197" s="66" t="n"/>
+      <c r="B197" s="9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C197" s="21" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/event-logs/{id}</t>
+        </is>
+      </c>
+      <c r="D197" s="21" t="inlineStr">
+        <is>
+          <t>Admin xem chi tiết toàn bộ raw JSON payload của sự kiện kỹ thuật</t>
+        </is>
+      </c>
+      <c r="E197" s="21" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Path:
+{
+  "id": "uuid"
+}</t>
+        </is>
+      </c>
+      <c r="F197" s="21" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "id": "uuid",
+  "eventId": "uuid",
+  "eventType": "OrderPaid",
+  "sourceService": "Commerce",
+  "actorId": "uuid",
+  "payload": {
+    "orderId": "uuid",
+    "totalAmount": 480000
+  },
+  "occurredAt": "2026-10-26T00:00:00Z",
+  "createdAt": "2026-10-26T00:00:00Z"
+}</t>
+        </is>
+      </c>
+      <c r="G197" s="21" t="inlineStr">
+        <is>
+          <t>401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.
+404 EVENT_LOG_NOT_FOUND: Event log entry was not found.</t>
+        </is>
+      </c>
+      <c r="H197" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-14</t>
+        </is>
+      </c>
       <c r="I197" s="21" t="n"/>
       <c r="J197" s="21" t="n"/>
       <c r="K197" s="21" t="n"/>
@@ -15730,13 +16397,65 @@
     </row>
     <row r="198" ht="15.75" customHeight="1" s="81">
       <c r="A198" s="76" t="n"/>
-      <c r="B198" s="76" t="n"/>
-      <c r="C198" s="77" t="n"/>
-      <c r="D198" s="77" t="n"/>
-      <c r="E198" s="77" t="n"/>
-      <c r="F198" s="77" t="n"/>
-      <c r="G198" s="77" t="n"/>
-      <c r="H198" s="66" t="n"/>
+      <c r="B198" s="76" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C198" s="77" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/health/broker</t>
+        </is>
+      </c>
+      <c r="D198" s="77" t="inlineStr">
+        <is>
+          <t>Admin theo dõi trạng thái sức khỏe, latency và queue depth RabbitMQ</t>
+        </is>
+      </c>
+      <c r="E198" s="77" t="inlineStr">
+        <is>
+          <t>Header:
+{
+  "Authorization": "Bearer &lt;JWT&gt;"
+}
+Query:
+{
+  "limit": 50
+}</t>
+        </is>
+      </c>
+      <c r="F198" s="77" t="inlineStr">
+        <is>
+          <t>200 OK:
+{
+  "currentStatus": "UP",
+  "lastCheckedAt": "2026-10-26T00:00:00Z",
+  "latestLatencyMs": 5,
+  "latestQueueDepth": 0,
+  "history": [
+    {
+      "id": "uuid",
+      "brokerName": "rabbitmq",
+      "status": "UP",
+      "latencyMs": 5,
+      "queueDepth": 0,
+      "checkedAt": "2026-10-26T00:00:00Z"
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G198" s="77" t="inlineStr">
+        <is>
+          <t>401 UNAUTHORIZED: Token is missing, expired, or invalid.
+403 FORBIDDEN: User does not have administrative permissions.</t>
+        </is>
+      </c>
+      <c r="H198" s="66" t="inlineStr">
+        <is>
+          <t>NOTI-16</t>
+        </is>
+      </c>
       <c r="I198" s="77" t="n"/>
       <c r="J198" s="77" t="n"/>
       <c r="K198" s="77" t="n"/>

</xml_diff>